<commit_message>
Feature: Add dashboard sorting options & resolve Windows CLI console unicode crash in compile_data.py
</commit_message>
<xml_diff>
--- a/assets/data/anime.xlsx
+++ b/assets/data/anime.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vedan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Anime Archive\assets\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5A8352F-7758-473F-B9D9-5666D313899F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560C9B4E-21BB-4DEF-80B9-3AA6DF7506EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Everything I Have Watched So Fa" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="174">
   <si>
     <t>Name</t>
   </si>
@@ -464,6 +464,84 @@
   </si>
   <si>
     <t>yes</t>
+  </si>
+  <si>
+    <t>N\A</t>
+  </si>
+  <si>
+    <t>A Silent Voice</t>
+  </si>
+  <si>
+    <t>聲の形 (Koe no Katachi)</t>
+  </si>
+  <si>
+    <t>Kyoto Animation</t>
+  </si>
+  <si>
+    <t>Naoko Yamada</t>
+  </si>
+  <si>
+    <t>Drama, Award Winning</t>
+  </si>
+  <si>
+    <t>silent-voice</t>
+  </si>
+  <si>
+    <t>Grave of the Fireflies</t>
+  </si>
+  <si>
+    <t>火垂るの墓 (Hotaru no Haka)</t>
+  </si>
+  <si>
+    <t>Drama</t>
+  </si>
+  <si>
+    <t>graves-of-the-fireflies</t>
+  </si>
+  <si>
+    <t>The Anthem of the Heart</t>
+  </si>
+  <si>
+    <t>心が叫びたがってるんだ。 (Kokoro ga Sakebitagatterunda.)</t>
+  </si>
+  <si>
+    <t>Tatsuyuki Nagai</t>
+  </si>
+  <si>
+    <t>anthem-of-the-heart</t>
+  </si>
+  <si>
+    <t>Attack on Titan</t>
+  </si>
+  <si>
+    <t>進撃の巨人 (Shingeki no Kyojin)</t>
+  </si>
+  <si>
+    <t>Wit Studio / MAPPA</t>
+  </si>
+  <si>
+    <t>Tetsuro Araki / Yuichiro Hayashi</t>
+  </si>
+  <si>
+    <t>Action, Drama, Suspense, Fantasy</t>
+  </si>
+  <si>
+    <t>attack-on-titan</t>
+  </si>
+  <si>
+    <t>A Lull in the Sea</t>
+  </si>
+  <si>
+    <t>凪のあすから (Nagi no Asukara)</t>
+  </si>
+  <si>
+    <t>P.A. Works</t>
+  </si>
+  <si>
+    <t>Toshiya Shinohara</t>
+  </si>
+  <si>
+    <t>lull-in-the-sea</t>
   </si>
 </sst>
 </file>
@@ -751,7 +829,7 @@
     <col min="8" max="8" width="22.85546875" customWidth="1"/>
     <col min="9" max="9" width="13.5703125" customWidth="1"/>
     <col min="11" max="11" width="20.85546875" customWidth="1"/>
-    <col min="12" max="12" width="20.28515625" style="4" customWidth="1"/>
+    <col min="12" max="12" width="28.28515625" style="4" customWidth="1"/>
     <col min="13" max="13" width="35.28515625" style="4" customWidth="1"/>
     <col min="14" max="14" width="12.5703125" style="4"/>
     <col min="15" max="15" width="26.140625" style="4" customWidth="1"/>
@@ -1641,7 +1719,7 @@
         <v>7.1</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>23</v>
+        <v>148</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>101</v>
@@ -1691,7 +1769,7 @@
         <v>7.25</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>23</v>
+        <v>148</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>107</v>
@@ -1823,59 +1901,244 @@
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
+      <c r="A22" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" s="3">
+        <v>8.94</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
+      <c r="G22" s="3">
+        <v>1</v>
+      </c>
+      <c r="H22" s="3">
+        <v>1</v>
+      </c>
+      <c r="I22" s="3">
+        <v>2016</v>
+      </c>
+      <c r="J22" s="3">
+        <v>130</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="M22" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="N22" s="4">
+        <v>21</v>
+      </c>
+      <c r="O22" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q22" s="4" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
+      <c r="A23" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B23" t="s">
+        <v>156</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" s="3">
+        <v>8.5</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
+      <c r="G23" s="3">
+        <v>1</v>
+      </c>
+      <c r="H23" s="3">
+        <v>1</v>
+      </c>
+      <c r="I23" s="3">
+        <v>1988</v>
+      </c>
+      <c r="J23" s="3">
+        <v>88</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="M23" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="N23" s="4">
+        <v>22</v>
+      </c>
+      <c r="O23" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="Q23" s="4" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
+      <c r="A24" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D24" s="3">
+        <v>8.02</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-      <c r="K24" s="3"/>
+      <c r="G24" s="3">
+        <v>1</v>
+      </c>
+      <c r="H24" s="3">
+        <v>1</v>
+      </c>
+      <c r="I24" s="3">
+        <v>2015</v>
+      </c>
+      <c r="J24" s="3">
+        <v>119</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="M24" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="N24" s="4">
+        <v>23</v>
+      </c>
+      <c r="O24" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q24" s="4" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
+      <c r="A25" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B25" t="s">
+        <v>164</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D25" s="3">
+        <v>8.7799999999999994</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
-      <c r="K25" s="3"/>
+      <c r="G25" s="3">
+        <v>4</v>
+      </c>
+      <c r="H25" s="3">
+        <v>22</v>
+      </c>
+      <c r="I25" s="3">
+        <v>2013</v>
+      </c>
+      <c r="J25" s="3">
+        <v>24</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="M25" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="N25" s="4">
+        <v>24</v>
+      </c>
+      <c r="O25" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="Q25" s="4" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
+      <c r="A26" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D26" s="3">
+        <v>8.06</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="3"/>
+      <c r="G26" s="3">
+        <v>1</v>
+      </c>
+      <c r="H26" s="3">
+        <v>26</v>
+      </c>
+      <c r="I26" s="3">
+        <v>2013</v>
+      </c>
+      <c r="J26" s="3">
+        <v>23</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="M26" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="N26" s="4">
+        <v>25</v>
+      </c>
+      <c r="O26" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q26" s="4" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C27" s="3"/>

</xml_diff>

<commit_message>
Update: Added 56 anime entries, reviews, and posters
</commit_message>
<xml_diff>
--- a/assets/data/anime.xlsx
+++ b/assets/data/anime.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Anime Archive\assets\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560C9B4E-21BB-4DEF-80B9-3AA6DF7506EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FC4C890-0E2F-405E-B763-6EFBD07759B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="335">
   <si>
     <t>Name</t>
   </si>
@@ -542,6 +542,489 @@
   </si>
   <si>
     <t>lull-in-the-sea</t>
+  </si>
+  <si>
+    <t>Hyouka</t>
+  </si>
+  <si>
+    <t>氷菓 (Hyouka)</t>
+  </si>
+  <si>
+    <t>Yasuhiro Takemoto</t>
+  </si>
+  <si>
+    <t>Mystery, Slice of Life</t>
+  </si>
+  <si>
+    <t>hyouka</t>
+  </si>
+  <si>
+    <t>Darling in the Franxx</t>
+  </si>
+  <si>
+    <t>ダーリン・イン・ザ・フランキス (Dārin In Za Furankisu)</t>
+  </si>
+  <si>
+    <t>A-1 Pictures / Trigger / CloverWorks</t>
+  </si>
+  <si>
+    <t>Atsushi Nishigori</t>
+  </si>
+  <si>
+    <t>Action, Drama, Sci-Fi, Romance</t>
+  </si>
+  <si>
+    <t>darling-in-the-franxx</t>
+  </si>
+  <si>
+    <t>Re:Zero</t>
+  </si>
+  <si>
+    <t>Re:ゼロから始める異世界生活 (Re:Zero kara Hajimeru Isekai Seikatsu)</t>
+  </si>
+  <si>
+    <t>White Fox</t>
+  </si>
+  <si>
+    <t>Masaharu Watanabe</t>
+  </si>
+  <si>
+    <t>Drama, Fantasy, Suspense</t>
+  </si>
+  <si>
+    <t>re-zero</t>
+  </si>
+  <si>
+    <t>Fireworks</t>
+  </si>
+  <si>
+    <t>打ち上げ花火、下から見るか？横から見るか？ (Uchiage Hanabi)</t>
+  </si>
+  <si>
+    <t>Shaft</t>
+  </si>
+  <si>
+    <t>Akiyuki Shinbo / Nobuyuki Takeuchi</t>
+  </si>
+  <si>
+    <t>fireworks</t>
+  </si>
+  <si>
+    <t>Hello World</t>
+  </si>
+  <si>
+    <t>HELLO WORLD</t>
+  </si>
+  <si>
+    <t>Graphinica</t>
+  </si>
+  <si>
+    <t>Tomohiko Itou</t>
+  </si>
+  <si>
+    <t>Sci-Fi, Drama, Romance</t>
+  </si>
+  <si>
+    <t>hello-world</t>
+  </si>
+  <si>
+    <t>Summer Ghost</t>
+  </si>
+  <si>
+    <t>サマーゴースト (Summer Ghost)</t>
+  </si>
+  <si>
+    <t>Flat Studio</t>
+  </si>
+  <si>
+    <t>loundraw</t>
+  </si>
+  <si>
+    <t>Drama, Supernatural</t>
+  </si>
+  <si>
+    <t>Look Back</t>
+  </si>
+  <si>
+    <t>ルックバック (Look Back)</t>
+  </si>
+  <si>
+    <t>Studio Durian</t>
+  </si>
+  <si>
+    <t>Kiyotaka Oshiyama</t>
+  </si>
+  <si>
+    <t>Drama, Avant Garde</t>
+  </si>
+  <si>
+    <t>Vinland Saga</t>
+  </si>
+  <si>
+    <t>ヴィンランド・サガ (Vinland Saga)</t>
+  </si>
+  <si>
+    <t>WIT Studio / MAPPA</t>
+  </si>
+  <si>
+    <t>Shuhei Yabuta</t>
+  </si>
+  <si>
+    <t>Action, Adventure, Drama</t>
+  </si>
+  <si>
+    <t>Death Note</t>
+  </si>
+  <si>
+    <t>デスノート (Death Note)</t>
+  </si>
+  <si>
+    <t>Madhouse</t>
+  </si>
+  <si>
+    <t>Tetsuro Araki</t>
+  </si>
+  <si>
+    <t>Supernatural, Suspense</t>
+  </si>
+  <si>
+    <t>Clannad</t>
+  </si>
+  <si>
+    <t>クラナド (Clannad)</t>
+  </si>
+  <si>
+    <t>Tatsuya Ishihara</t>
+  </si>
+  <si>
+    <t>Insomniacs After School</t>
+  </si>
+  <si>
+    <t>君は放課後インソムニア (Kimi wa Houkago Insomnia)</t>
+  </si>
+  <si>
+    <t>LIDENFILMS</t>
+  </si>
+  <si>
+    <t>Yuki Ikeda</t>
+  </si>
+  <si>
+    <t>Romance, Slice of Life</t>
+  </si>
+  <si>
+    <t>The Apothecary Diaries</t>
+  </si>
+  <si>
+    <t>薬屋のひとりごと (Kusuriya no Hitorigoto)</t>
+  </si>
+  <si>
+    <t>OLM / TOHO animation</t>
+  </si>
+  <si>
+    <t>Norihiro Naganuma</t>
+  </si>
+  <si>
+    <t>Drama, Mystery, Medical</t>
+  </si>
+  <si>
+    <t>Jujutsu Kaisen</t>
+  </si>
+  <si>
+    <t>呪術廻戦 (Jujutsu Kaisen)</t>
+  </si>
+  <si>
+    <t>MAPPA</t>
+  </si>
+  <si>
+    <t>Sunghoo Park / Shota Goshozono</t>
+  </si>
+  <si>
+    <t>Anohana</t>
+  </si>
+  <si>
+    <t>あの日見た花の名前を僕達はまだ知らない。 (Anohana)</t>
+  </si>
+  <si>
+    <t>365 Days to the Wedding</t>
+  </si>
+  <si>
+    <t>Ashi Productions</t>
+  </si>
+  <si>
+    <t>Hiroshi Ikehata</t>
+  </si>
+  <si>
+    <t>Blue Box</t>
+  </si>
+  <si>
+    <t>アオのハコ (Ao no Hako)</t>
+  </si>
+  <si>
+    <t>Telecom Animation Film</t>
+  </si>
+  <si>
+    <t>Yūichirō Yano</t>
+  </si>
+  <si>
+    <t>Romance, Sports</t>
+  </si>
+  <si>
+    <t>The Angel Next Door Spoils Me Rotten</t>
+  </si>
+  <si>
+    <t>お隣の天使様にいつの間にか駄目人間にされていた件 (Otonari no Tenshi-sama)</t>
+  </si>
+  <si>
+    <t>Project No.9</t>
+  </si>
+  <si>
+    <t>Lihua Wang / Chihiro Kumano</t>
+  </si>
+  <si>
+    <t>The Dangers in My Heart</t>
+  </si>
+  <si>
+    <t>僕の心のヤバイやつ (Boku no Kokoro no Yabai Yatsu)</t>
+  </si>
+  <si>
+    <t>Shin-Ei Animation</t>
+  </si>
+  <si>
+    <t>Hiroaki Akagi</t>
+  </si>
+  <si>
+    <t>Comedy, Romance</t>
+  </si>
+  <si>
+    <t>Studio Mother</t>
+  </si>
+  <si>
+    <t>Junichi Yamamoto / Takao Kato</t>
+  </si>
+  <si>
+    <t>Kaguya-sama: Love Is War</t>
+  </si>
+  <si>
+    <t>かぐや様は告らせたい ～天才たちの恋愛頭脳戦～ (Kaguya-sama wa Kokurasetai)</t>
+  </si>
+  <si>
+    <t>Shinichi Omata</t>
+  </si>
+  <si>
+    <t>Toradora!</t>
+  </si>
+  <si>
+    <t>とらドラ！ (Toradora!)</t>
+  </si>
+  <si>
+    <t>J.C.Staff</t>
+  </si>
+  <si>
+    <t>Comedy, Drama, Romance</t>
+  </si>
+  <si>
+    <t>Erased</t>
+  </si>
+  <si>
+    <t>僕だけがいない街 (Boku dake ga Inai Machi)</t>
+  </si>
+  <si>
+    <t>Mystery, Supernatural, Suspense</t>
+  </si>
+  <si>
+    <t>Classroom of the Elite</t>
+  </si>
+  <si>
+    <t>ようこそ実力至上主義の教室へ (Youkoso Jitsuryoku Shijou Shugi no Kyrosshitsu e)</t>
+  </si>
+  <si>
+    <t>Lerche</t>
+  </si>
+  <si>
+    <t>Seiji Kishi / Hiroyuki Hashimoto / Noriyuki Nomata</t>
+  </si>
+  <si>
+    <t>Drama, Suspense</t>
+  </si>
+  <si>
+    <t>Spy × Family</t>
+  </si>
+  <si>
+    <t>SPY×FAMILY (Spy × Family)</t>
+  </si>
+  <si>
+    <t>Wit Studio / CloverWorks</t>
+  </si>
+  <si>
+    <t>Kazuhiro Furuhashi</t>
+  </si>
+  <si>
+    <t>Action, Comedy</t>
+  </si>
+  <si>
+    <t>Alya Sometimes Hides Her Feelings in Russian</t>
+  </si>
+  <si>
+    <t>時々ボソッとロシア語でデレる隣のアーlyaさん (Tokidoki Bosotto Russia-go de Dereru Tonari no Alya-san)</t>
+  </si>
+  <si>
+    <t>Doga Kobo</t>
+  </si>
+  <si>
+    <t>Ryota Itoh</t>
+  </si>
+  <si>
+    <t>The Fragrant Flower Blooms with Dignity</t>
+  </si>
+  <si>
+    <t>薫る花は凛と咲く (Kaoru Hana wa Rin to Saku)</t>
+  </si>
+  <si>
+    <t>Miho Tan Tanaka</t>
+  </si>
+  <si>
+    <t>Howl's Moving Castle</t>
+  </si>
+  <si>
+    <t>ハウルの動く城 (Hauru no Ugoku Shiro)</t>
+  </si>
+  <si>
+    <t>Hayao Miyazaki</t>
+  </si>
+  <si>
+    <t>Adventure, Fantasy, Romance</t>
+  </si>
+  <si>
+    <t>Chainsaw Man</t>
+  </si>
+  <si>
+    <t>チェンソーマン (Chainsaw Man)</t>
+  </si>
+  <si>
+    <t>Ryu Nakayama / Tatsuya Yoshihara</t>
+  </si>
+  <si>
+    <t>Action, Dark Fantasy, Gore</t>
+  </si>
+  <si>
+    <t>Too Many Losing Heroines!</t>
+  </si>
+  <si>
+    <t>負けヒロインが多すぎる！ (Make Heroine ga Oosugiru!)</t>
+  </si>
+  <si>
+    <t>Shotaro Kitamura</t>
+  </si>
+  <si>
+    <t>ジョゼと虎と魚たち (Joze to Tora to Sakana-tachi)</t>
+  </si>
+  <si>
+    <t>Bones</t>
+  </si>
+  <si>
+    <t>Kotaro Tamura</t>
+  </si>
+  <si>
+    <t>More Than a Married Couple,  But Not Lovers</t>
+  </si>
+  <si>
+    <t>夫婦以上、恋人未満。 (Fuufu Ijou Koibito Miman.)</t>
+  </si>
+  <si>
+    <t>結婚するって、本当ですか (Kekkon Surutte,  Honto desu ka?)</t>
+  </si>
+  <si>
+    <t>Josee,  the Tiger and the Fish</t>
+  </si>
+  <si>
+    <t>summer-ghost</t>
+  </si>
+  <si>
+    <t>look-back</t>
+  </si>
+  <si>
+    <t>vinland-saga</t>
+  </si>
+  <si>
+    <t>death-note</t>
+  </si>
+  <si>
+    <t>jujutsu-kaisen</t>
+  </si>
+  <si>
+    <t>blue-box</t>
+  </si>
+  <si>
+    <t>spy-family</t>
+  </si>
+  <si>
+    <t>chainsaw-man</t>
+  </si>
+  <si>
+    <t>clannad</t>
+  </si>
+  <si>
+    <t>insomniacs-after-school</t>
+  </si>
+  <si>
+    <t>classroom-of-the-elite</t>
+  </si>
+  <si>
+    <t>the-fragrant-flower-blooms-with-dignity</t>
+  </si>
+  <si>
+    <t>josee-the-tiger-and-the-fish</t>
+  </si>
+  <si>
+    <t>anohana</t>
+  </si>
+  <si>
+    <t>days-to-the-wedding</t>
+  </si>
+  <si>
+    <t>the-apothecary-diaries</t>
+  </si>
+  <si>
+    <t>the-dangers-in-my-heart</t>
+  </si>
+  <si>
+    <t>more-than-a-married-couple-but-not-lovers</t>
+  </si>
+  <si>
+    <t>erased</t>
+  </si>
+  <si>
+    <t>alya-sometimes-hides-her-feelings-in-russian</t>
+  </si>
+  <si>
+    <t>howl's-moving-castle</t>
+  </si>
+  <si>
+    <t>the-angel-next-door-spoils-me-rotten</t>
+  </si>
+  <si>
+    <t>kaguya-sama-love-is-war</t>
+  </si>
+  <si>
+    <t>toradora</t>
+  </si>
+  <si>
+    <t>too-many-losing-heroines</t>
+  </si>
+  <si>
+    <t>Takopi's Original Sin</t>
+  </si>
+  <si>
+    <t>タコピーの原罪 (Takopi no Genzai)</t>
+  </si>
+  <si>
+    <t>Shinpei Tomooka</t>
+  </si>
+  <si>
+    <t>Drama, Psychological, Sci-Fi</t>
+  </si>
+  <si>
+    <t>takopi's-original-sin</t>
   </si>
 </sst>
 </file>
@@ -589,7 +1072,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -600,6 +1083,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -824,15 +1310,17 @@
   <cols>
     <col min="1" max="1" width="41.28515625" customWidth="1"/>
     <col min="2" max="2" width="95.28515625" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" style="4"/>
     <col min="6" max="6" width="31.42578125" customWidth="1"/>
     <col min="7" max="7" width="18.42578125" customWidth="1"/>
     <col min="8" max="8" width="22.85546875" customWidth="1"/>
     <col min="9" max="9" width="13.5703125" customWidth="1"/>
-    <col min="11" max="11" width="20.85546875" customWidth="1"/>
-    <col min="12" max="12" width="28.28515625" style="4" customWidth="1"/>
-    <col min="13" max="13" width="35.28515625" style="4" customWidth="1"/>
+    <col min="11" max="11" width="35.42578125" customWidth="1"/>
+    <col min="12" max="12" width="31.7109375" style="4" customWidth="1"/>
+    <col min="13" max="13" width="36.7109375" style="4" customWidth="1"/>
     <col min="14" max="14" width="12.5703125" style="4"/>
-    <col min="15" max="15" width="26.140625" style="4" customWidth="1"/>
+    <col min="15" max="15" width="40.42578125" style="4" customWidth="1"/>
     <col min="16" max="16" width="15.5703125" customWidth="1"/>
     <col min="17" max="17" width="12.5703125" style="4"/>
   </cols>
@@ -2141,347 +2629,1493 @@
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
+      <c r="A27" t="s">
+        <v>174</v>
+      </c>
+      <c r="B27" t="s">
+        <v>175</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D27" s="3">
+        <v>8.08</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
-      <c r="K27" s="3"/>
+      <c r="G27" s="3">
+        <v>1</v>
+      </c>
+      <c r="H27" s="3">
+        <v>22</v>
+      </c>
+      <c r="I27" s="3">
+        <v>2012</v>
+      </c>
+      <c r="J27" s="3">
+        <v>25</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="M27" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="N27" s="4">
+        <v>26</v>
+      </c>
+      <c r="O27" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q27" s="4" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
+      <c r="A28" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B28" t="s">
+        <v>180</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D28" s="3">
+        <v>7.2</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
-      <c r="K28" s="3"/>
+      <c r="G28" s="3">
+        <v>1</v>
+      </c>
+      <c r="H28" s="3">
+        <v>24</v>
+      </c>
+      <c r="I28" s="3">
+        <v>2018</v>
+      </c>
+      <c r="J28" s="3">
+        <v>24</v>
+      </c>
+      <c r="K28" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="L28" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="M28" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="N28" s="4">
+        <v>27</v>
+      </c>
+      <c r="O28" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q28" s="4" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
+      <c r="A29" t="s">
+        <v>185</v>
+      </c>
+      <c r="B29" t="s">
+        <v>186</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D29" s="3">
+        <v>8.24</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F29" s="3"/>
-      <c r="G29" s="3"/>
-      <c r="H29" s="3"/>
-      <c r="I29" s="3"/>
-      <c r="J29" s="3"/>
-      <c r="K29" s="3"/>
+      <c r="G29" s="3">
+        <v>3</v>
+      </c>
+      <c r="H29" s="3">
+        <v>25</v>
+      </c>
+      <c r="I29" s="3">
+        <v>2016</v>
+      </c>
+      <c r="J29" s="3">
+        <v>25</v>
+      </c>
+      <c r="K29" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="L29" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="M29" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="N29" s="4">
+        <v>28</v>
+      </c>
+      <c r="O29" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q29" s="4" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
+      <c r="A30" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B30" t="s">
+        <v>192</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D30" s="3">
+        <v>6.6</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F30" s="3"/>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
-      <c r="J30" s="3"/>
-      <c r="K30" s="3"/>
+      <c r="G30" s="3">
+        <v>1</v>
+      </c>
+      <c r="H30" s="3">
+        <v>1</v>
+      </c>
+      <c r="I30" s="3">
+        <v>2017</v>
+      </c>
+      <c r="J30" s="3">
+        <v>90</v>
+      </c>
+      <c r="K30" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="L30" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="M30" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="N30" s="4">
+        <v>29</v>
+      </c>
+      <c r="O30" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q30" s="4" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
+      <c r="A31" t="s">
+        <v>196</v>
+      </c>
+      <c r="B31" t="s">
+        <v>197</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" s="3">
+        <v>7.55</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
-      <c r="I31" s="3"/>
-      <c r="J31" s="3"/>
-      <c r="K31" s="3"/>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
-      <c r="I32" s="3"/>
-      <c r="J32" s="3"/>
-      <c r="K32" s="3"/>
-    </row>
-    <row r="33" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
+      <c r="G31" s="3">
+        <v>1</v>
+      </c>
+      <c r="H31" s="3">
+        <v>1</v>
+      </c>
+      <c r="I31" s="3">
+        <v>2019</v>
+      </c>
+      <c r="J31" s="3">
+        <v>98</v>
+      </c>
+      <c r="K31" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="L31" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="M31" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="N31" s="4">
+        <v>30</v>
+      </c>
+      <c r="O31" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="Q31" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B32" t="s">
+        <v>203</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D32" s="4">
+        <v>7.42</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G32" s="4">
+        <v>1</v>
+      </c>
+      <c r="H32" s="4">
+        <v>1</v>
+      </c>
+      <c r="I32" s="4">
+        <v>2021</v>
+      </c>
+      <c r="J32" s="4">
+        <v>40</v>
+      </c>
+      <c r="K32" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="L32" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="M32" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="N32" s="4">
+        <v>31</v>
+      </c>
+      <c r="O32" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="Q32" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>207</v>
+      </c>
+      <c r="B33" t="s">
+        <v>208</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="3">
+        <v>8.75</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
-      <c r="J33" s="3"/>
-      <c r="K33" s="3"/>
-    </row>
-    <row r="34" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
+      <c r="G33" s="3">
+        <v>1</v>
+      </c>
+      <c r="H33" s="3">
+        <v>1</v>
+      </c>
+      <c r="I33" s="3">
+        <v>2024</v>
+      </c>
+      <c r="J33" s="3">
+        <v>58</v>
+      </c>
+      <c r="K33" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="L33" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="M33" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="N33" s="4">
+        <v>32</v>
+      </c>
+      <c r="O33" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="Q33" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>212</v>
+      </c>
+      <c r="B34" t="s">
+        <v>213</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D34" s="3">
+        <v>8.75</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F34" s="3"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
-      <c r="I34" s="3"/>
-      <c r="J34" s="3"/>
-      <c r="K34" s="3"/>
-    </row>
-    <row r="35" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
+      <c r="G34" s="3">
+        <v>2</v>
+      </c>
+      <c r="H34" s="3">
+        <v>24</v>
+      </c>
+      <c r="I34" s="3">
+        <v>2019</v>
+      </c>
+      <c r="J34" s="3">
+        <v>24</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="L34" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="M34" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="N34" s="4">
+        <v>33</v>
+      </c>
+      <c r="O34" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="Q34" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>217</v>
+      </c>
+      <c r="B35" t="s">
+        <v>218</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D35" s="3">
+        <v>8.6199999999999992</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F35" s="3"/>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
-      <c r="I35" s="3"/>
-      <c r="J35" s="3"/>
-      <c r="K35" s="3"/>
-    </row>
-    <row r="36" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
+      <c r="G35" s="3">
+        <v>1</v>
+      </c>
+      <c r="H35" s="3">
+        <v>37</v>
+      </c>
+      <c r="I35" s="3">
+        <v>2006</v>
+      </c>
+      <c r="J35" s="3">
+        <v>23</v>
+      </c>
+      <c r="K35" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="L35" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="M35" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="N35" s="4">
+        <v>34</v>
+      </c>
+      <c r="O35" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="Q35" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>222</v>
+      </c>
+      <c r="B36" t="s">
+        <v>223</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D36" s="3">
+        <v>8.01</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F36" s="3"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-      <c r="I36" s="3"/>
-      <c r="J36" s="3"/>
-      <c r="K36" s="3"/>
-    </row>
-    <row r="37" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
+      <c r="G36" s="3">
+        <v>2</v>
+      </c>
+      <c r="H36" s="3">
+        <v>23</v>
+      </c>
+      <c r="I36" s="3">
+        <v>2007</v>
+      </c>
+      <c r="J36" s="3">
+        <v>24</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="L36" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="M36" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="N36" s="4">
+        <v>35</v>
+      </c>
+      <c r="O36" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="Q36" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>225</v>
+      </c>
+      <c r="B37" t="s">
+        <v>226</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D37" s="3">
+        <v>8.02</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
-      <c r="I37" s="3"/>
-      <c r="J37" s="3"/>
-      <c r="K37" s="3"/>
-    </row>
-    <row r="38" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C38" s="3"/>
-      <c r="D38" s="3"/>
-      <c r="E38" s="3"/>
+      <c r="G37" s="3">
+        <v>1</v>
+      </c>
+      <c r="H37" s="3">
+        <v>13</v>
+      </c>
+      <c r="I37" s="3">
+        <v>2023</v>
+      </c>
+      <c r="J37" s="3">
+        <v>24</v>
+      </c>
+      <c r="K37" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="L37" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="M37" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="N37" s="4">
+        <v>36</v>
+      </c>
+      <c r="O37" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="Q37" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>230</v>
+      </c>
+      <c r="B38" t="s">
+        <v>231</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D38" s="3">
+        <v>8.9</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F38" s="3"/>
-      <c r="G38" s="3"/>
-      <c r="H38" s="3"/>
-      <c r="I38" s="3"/>
-      <c r="J38" s="3"/>
-      <c r="K38" s="3"/>
-    </row>
-    <row r="39" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
+      <c r="G38" s="3">
+        <v>2</v>
+      </c>
+      <c r="H38" s="3">
+        <v>24</v>
+      </c>
+      <c r="I38" s="3">
+        <v>2023</v>
+      </c>
+      <c r="J38" s="3">
+        <v>24</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="L38" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="M38" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="N38" s="4">
+        <v>37</v>
+      </c>
+      <c r="O38" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="Q38" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>235</v>
+      </c>
+      <c r="B39" t="s">
+        <v>236</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D39" s="3">
+        <v>8.65</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F39" s="3"/>
-      <c r="G39" s="3"/>
-      <c r="H39" s="3"/>
-      <c r="I39" s="3"/>
-      <c r="J39" s="3"/>
-      <c r="K39" s="3"/>
-    </row>
-    <row r="40" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
+      <c r="G39" s="3">
+        <v>2</v>
+      </c>
+      <c r="H39" s="3">
+        <v>24</v>
+      </c>
+      <c r="I39" s="3">
+        <v>2020</v>
+      </c>
+      <c r="J39" s="3">
+        <v>24</v>
+      </c>
+      <c r="K39" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="L39" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="M39" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="N39" s="4">
+        <v>38</v>
+      </c>
+      <c r="O39" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="Q39" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>239</v>
+      </c>
+      <c r="B40" t="s">
+        <v>240</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D40" s="3">
+        <v>8.31</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F40" s="3"/>
-      <c r="G40" s="3"/>
-      <c r="H40" s="3"/>
-      <c r="I40" s="3"/>
-      <c r="J40" s="3"/>
-      <c r="K40" s="3"/>
-    </row>
-    <row r="41" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C41" s="3"/>
-      <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
+      <c r="G40" s="3">
+        <v>1</v>
+      </c>
+      <c r="H40" s="3">
+        <v>11</v>
+      </c>
+      <c r="I40" s="3">
+        <v>2011</v>
+      </c>
+      <c r="J40" s="3">
+        <v>22</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="L40" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="M40" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="N40" s="4">
+        <v>39</v>
+      </c>
+      <c r="O40" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="Q40" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>241</v>
+      </c>
+      <c r="B41" t="s">
+        <v>303</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D41" s="3">
+        <v>7.22</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F41" s="3"/>
-      <c r="G41" s="3"/>
-      <c r="H41" s="3"/>
-      <c r="I41" s="3"/>
-      <c r="J41" s="3"/>
-      <c r="K41" s="3"/>
-    </row>
-    <row r="42" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
+      <c r="G41" s="3">
+        <v>1</v>
+      </c>
+      <c r="H41" s="3">
+        <v>12</v>
+      </c>
+      <c r="I41" s="3">
+        <v>2024</v>
+      </c>
+      <c r="J41" s="3">
+        <v>24</v>
+      </c>
+      <c r="K41" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="L41" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="M41" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="N41" s="4">
+        <v>40</v>
+      </c>
+      <c r="O41" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="Q41" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>244</v>
+      </c>
+      <c r="B42" t="s">
+        <v>245</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D42" s="3">
+        <v>8.35</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F42" s="3"/>
-      <c r="G42" s="3"/>
-      <c r="H42" s="3"/>
-      <c r="I42" s="3"/>
-      <c r="J42" s="3"/>
-      <c r="K42" s="3"/>
-    </row>
-    <row r="43" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C43" s="3"/>
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
+      <c r="G42" s="3">
+        <v>2</v>
+      </c>
+      <c r="H42" s="3">
+        <v>25</v>
+      </c>
+      <c r="I42" s="3">
+        <v>2024</v>
+      </c>
+      <c r="J42" s="3">
+        <v>24</v>
+      </c>
+      <c r="K42" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="L42" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="M42" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="N42" s="4">
+        <v>41</v>
+      </c>
+      <c r="O42" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="Q42" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>249</v>
+      </c>
+      <c r="B43" t="s">
+        <v>250</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D43" s="3">
+        <v>7.85</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F43" s="3"/>
-      <c r="G43" s="3"/>
-      <c r="H43" s="3"/>
-      <c r="I43" s="3"/>
-      <c r="J43" s="3"/>
-      <c r="K43" s="3"/>
-    </row>
-    <row r="44" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C44" s="3"/>
-      <c r="D44" s="3"/>
-      <c r="E44" s="3"/>
+      <c r="G43" s="3">
+        <v>2</v>
+      </c>
+      <c r="H43" s="3">
+        <v>12</v>
+      </c>
+      <c r="I43" s="3">
+        <v>2023</v>
+      </c>
+      <c r="J43" s="3">
+        <v>24</v>
+      </c>
+      <c r="K43" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="L43" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="M43" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="N43" s="4">
+        <v>42</v>
+      </c>
+      <c r="O43" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="Q43" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>253</v>
+      </c>
+      <c r="B44" t="s">
+        <v>254</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D44" s="3">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F44" s="3"/>
-      <c r="G44" s="3"/>
-      <c r="H44" s="3"/>
-      <c r="I44" s="3"/>
-      <c r="J44" s="3"/>
-      <c r="K44" s="3"/>
-    </row>
-    <row r="45" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
+      <c r="G44" s="3">
+        <v>2</v>
+      </c>
+      <c r="H44" s="3">
+        <v>12</v>
+      </c>
+      <c r="I44" s="3">
+        <v>2023</v>
+      </c>
+      <c r="J44" s="3">
+        <v>24</v>
+      </c>
+      <c r="K44" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="L44" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="M44" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="N44" s="4">
+        <v>43</v>
+      </c>
+      <c r="O44" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="Q44" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>301</v>
+      </c>
+      <c r="B45" t="s">
+        <v>302</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D45" s="3">
+        <v>7.51</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F45" s="3"/>
-      <c r="G45" s="3"/>
-      <c r="H45" s="3"/>
-      <c r="I45" s="3"/>
-      <c r="J45" s="3"/>
-      <c r="K45" s="3"/>
-    </row>
-    <row r="46" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C46" s="3"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
+      <c r="G45" s="3">
+        <v>1</v>
+      </c>
+      <c r="H45" s="3">
+        <v>12</v>
+      </c>
+      <c r="I45" s="3">
+        <v>2022</v>
+      </c>
+      <c r="J45" s="4">
+        <v>24</v>
+      </c>
+      <c r="K45" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="L45" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="M45" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="N45" s="4">
+        <v>44</v>
+      </c>
+      <c r="O45" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="Q45" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>260</v>
+      </c>
+      <c r="B46" t="s">
+        <v>261</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D46" s="3">
+        <v>8.75</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F46" s="3"/>
-      <c r="G46" s="3"/>
-      <c r="H46" s="3"/>
-      <c r="I46" s="3"/>
-      <c r="J46" s="3"/>
-      <c r="K46" s="3"/>
-    </row>
-    <row r="47" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
+      <c r="G46" s="3">
+        <v>3</v>
+      </c>
+      <c r="H46" s="3">
+        <v>12</v>
+      </c>
+      <c r="I46" s="3">
+        <v>2019</v>
+      </c>
+      <c r="J46" s="3">
+        <v>24</v>
+      </c>
+      <c r="K46" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="L46" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="M46" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="N46" s="4">
+        <v>45</v>
+      </c>
+      <c r="O46" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="Q46" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>263</v>
+      </c>
+      <c r="B47" t="s">
+        <v>264</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D47" s="3">
+        <v>8.1</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
-      <c r="H47" s="3"/>
-      <c r="I47" s="3"/>
-      <c r="J47" s="3"/>
-      <c r="K47" s="3"/>
-    </row>
-    <row r="48" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
+      <c r="G47" s="3">
+        <v>1</v>
+      </c>
+      <c r="H47" s="3">
+        <v>25</v>
+      </c>
+      <c r="I47" s="3">
+        <v>2008</v>
+      </c>
+      <c r="J47" s="3">
+        <v>24</v>
+      </c>
+      <c r="K47" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="L47" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="M47" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="N47" s="4">
+        <v>46</v>
+      </c>
+      <c r="O47" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="Q47" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>267</v>
+      </c>
+      <c r="B48" t="s">
+        <v>268</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D48" s="3">
+        <v>8.31</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F48" s="3"/>
-      <c r="G48" s="3"/>
-      <c r="H48" s="3"/>
-      <c r="I48" s="3"/>
-      <c r="J48" s="3"/>
-      <c r="K48" s="3"/>
-    </row>
-    <row r="49" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C49" s="3"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
+      <c r="G48" s="3">
+        <v>1</v>
+      </c>
+      <c r="H48" s="3">
+        <v>12</v>
+      </c>
+      <c r="I48" s="3">
+        <v>2016</v>
+      </c>
+      <c r="J48" s="3">
+        <v>23</v>
+      </c>
+      <c r="K48" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="L48" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="M48" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="N48" s="4">
+        <v>47</v>
+      </c>
+      <c r="O48" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="Q48" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>270</v>
+      </c>
+      <c r="B49" t="s">
+        <v>271</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D49" s="3">
+        <v>7.86</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F49" s="3"/>
-      <c r="G49" s="3"/>
-      <c r="H49" s="3"/>
-      <c r="I49" s="3"/>
-      <c r="J49" s="3"/>
-      <c r="K49" s="3"/>
-    </row>
-    <row r="50" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C50" s="3"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
+      <c r="G49" s="3">
+        <v>4</v>
+      </c>
+      <c r="H49" s="3">
+        <v>13</v>
+      </c>
+      <c r="I49" s="3">
+        <v>2017</v>
+      </c>
+      <c r="J49" s="3">
+        <v>24</v>
+      </c>
+      <c r="K49" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="L49" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="M49" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="N49" s="4">
+        <v>48</v>
+      </c>
+      <c r="O49" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="Q49" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>275</v>
+      </c>
+      <c r="B50" t="s">
+        <v>276</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D50" s="3">
+        <v>8.5</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F50" s="3"/>
-      <c r="G50" s="3"/>
-      <c r="H50" s="3"/>
-      <c r="I50" s="3"/>
-      <c r="J50" s="3"/>
-      <c r="K50" s="3"/>
-    </row>
-    <row r="51" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C51" s="3"/>
-      <c r="D51" s="3"/>
-      <c r="E51" s="3"/>
+      <c r="G50" s="3">
+        <v>3</v>
+      </c>
+      <c r="H50" s="3">
+        <v>12</v>
+      </c>
+      <c r="I50" s="3">
+        <v>2022</v>
+      </c>
+      <c r="J50" s="3">
+        <v>24</v>
+      </c>
+      <c r="K50" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="L50" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="M50" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="N50" s="4">
+        <v>49</v>
+      </c>
+      <c r="O50" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="Q50" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>280</v>
+      </c>
+      <c r="B51" t="s">
+        <v>281</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D51" s="3">
+        <v>7.62</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F51" s="3"/>
-      <c r="G51" s="3"/>
-      <c r="H51" s="3"/>
-      <c r="I51" s="3"/>
-      <c r="J51" s="3"/>
-      <c r="K51" s="3"/>
-    </row>
-    <row r="52" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
+      <c r="G51" s="3">
+        <v>2</v>
+      </c>
+      <c r="H51" s="3">
+        <v>12</v>
+      </c>
+      <c r="I51" s="3">
+        <v>2024</v>
+      </c>
+      <c r="J51" s="3">
+        <v>24</v>
+      </c>
+      <c r="K51" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="L51" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="M51" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="N51" s="4">
+        <v>50</v>
+      </c>
+      <c r="O51" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="Q51" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>284</v>
+      </c>
+      <c r="B52" t="s">
+        <v>285</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D52" s="3">
+        <v>8.42</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F52" s="3"/>
-      <c r="G52" s="3"/>
-      <c r="H52" s="3"/>
-      <c r="I52" s="3"/>
-      <c r="J52" s="3"/>
-      <c r="K52" s="3"/>
-    </row>
-    <row r="53" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C53" s="3"/>
-      <c r="D53" s="3"/>
-      <c r="E53" s="3"/>
+      <c r="G52" s="3">
+        <v>1</v>
+      </c>
+      <c r="H52" s="3">
+        <v>12</v>
+      </c>
+      <c r="I52" s="3">
+        <v>2026</v>
+      </c>
+      <c r="J52" s="3">
+        <v>24</v>
+      </c>
+      <c r="K52" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L52" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="M52" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="N52" s="4">
+        <v>51</v>
+      </c>
+      <c r="O52" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="Q52" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>287</v>
+      </c>
+      <c r="B53" t="s">
+        <v>288</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D53" s="3">
+        <v>8.66</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F53" s="3"/>
-      <c r="G53" s="3"/>
-      <c r="H53" s="3"/>
-      <c r="I53" s="3"/>
-      <c r="J53" s="3"/>
-      <c r="K53" s="3"/>
-    </row>
-    <row r="54" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C54" s="3"/>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
+      <c r="G53" s="3">
+        <v>1</v>
+      </c>
+      <c r="H53" s="3">
+        <v>1</v>
+      </c>
+      <c r="I53" s="3">
+        <v>2004</v>
+      </c>
+      <c r="J53" s="3">
+        <v>119</v>
+      </c>
+      <c r="K53" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="L53" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="M53" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="N53" s="4">
+        <v>52</v>
+      </c>
+      <c r="O53" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="Q53" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>291</v>
+      </c>
+      <c r="B54" t="s">
+        <v>292</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D54" s="3">
+        <v>8.51</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F54" s="3"/>
-      <c r="G54" s="3"/>
-      <c r="H54" s="3"/>
-      <c r="I54" s="3"/>
-      <c r="J54" s="3"/>
-      <c r="K54" s="3"/>
-    </row>
-    <row r="55" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C55" s="3"/>
-      <c r="D55" s="3"/>
-      <c r="E55" s="3"/>
+      <c r="G54" s="3">
+        <v>2</v>
+      </c>
+      <c r="H54" s="3">
+        <v>12</v>
+      </c>
+      <c r="I54" s="3">
+        <v>2022</v>
+      </c>
+      <c r="J54" s="3">
+        <v>24</v>
+      </c>
+      <c r="K54" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="L54" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="M54" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="N54" s="4">
+        <v>53</v>
+      </c>
+      <c r="O54" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="Q54" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>295</v>
+      </c>
+      <c r="B55" t="s">
+        <v>296</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D55" s="3">
+        <v>8.25</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F55" s="3"/>
-      <c r="G55" s="3"/>
-      <c r="H55" s="3"/>
-      <c r="I55" s="3"/>
-      <c r="J55" s="3"/>
-      <c r="K55" s="3"/>
-    </row>
-    <row r="56" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C56" s="3"/>
-      <c r="D56" s="3"/>
-      <c r="E56" s="3"/>
+      <c r="G55" s="3">
+        <v>1</v>
+      </c>
+      <c r="H55" s="3">
+        <v>12</v>
+      </c>
+      <c r="I55" s="3">
+        <v>2024</v>
+      </c>
+      <c r="J55" s="3">
+        <v>24</v>
+      </c>
+      <c r="K55" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="L55" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="M55" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="N55" s="4">
+        <v>54</v>
+      </c>
+      <c r="O55" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="Q55" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>304</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D56" s="3">
+        <v>8.41</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F56" s="3"/>
-      <c r="G56" s="3"/>
-      <c r="H56" s="3"/>
-      <c r="I56" s="3"/>
-      <c r="J56" s="3"/>
-      <c r="K56" s="3"/>
-    </row>
-    <row r="57" spans="3:11" x14ac:dyDescent="0.2">
-      <c r="C57" s="3"/>
-      <c r="D57" s="3"/>
-      <c r="E57" s="3"/>
+      <c r="G56" s="3">
+        <v>1</v>
+      </c>
+      <c r="H56" s="3">
+        <v>1</v>
+      </c>
+      <c r="I56" s="3">
+        <v>2020</v>
+      </c>
+      <c r="J56" s="3">
+        <v>98</v>
+      </c>
+      <c r="K56" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="L56" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="M56" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="N56" s="4">
+        <v>55</v>
+      </c>
+      <c r="O56" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="Q56" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>330</v>
+      </c>
+      <c r="B57" t="s">
+        <v>331</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D57" s="3">
+        <v>7.94</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="F57" s="3"/>
-      <c r="G57" s="3"/>
-      <c r="H57" s="3"/>
-      <c r="I57" s="3"/>
-      <c r="J57" s="3"/>
-      <c r="K57" s="3"/>
-    </row>
-    <row r="58" spans="3:11" x14ac:dyDescent="0.2">
+      <c r="G57" s="3">
+        <v>1</v>
+      </c>
+      <c r="H57" s="3">
+        <v>8</v>
+      </c>
+      <c r="I57" s="3">
+        <v>2026</v>
+      </c>
+      <c r="J57" s="3">
+        <v>24</v>
+      </c>
+      <c r="K57" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L57" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="M57" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="N57" s="4">
+        <v>56</v>
+      </c>
+      <c r="O57" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="Q57" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
       <c r="E58" s="3"/>
@@ -2492,7 +4126,7 @@
       <c r="J58" s="3"/>
       <c r="K58" s="3"/>
     </row>
-    <row r="59" spans="3:11" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
       <c r="E59" s="3"/>
@@ -2503,7 +4137,7 @@
       <c r="J59" s="3"/>
       <c r="K59" s="3"/>
     </row>
-    <row r="60" spans="3:11" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
       <c r="E60" s="3"/>
@@ -2514,7 +4148,7 @@
       <c r="J60" s="3"/>
       <c r="K60" s="3"/>
     </row>
-    <row r="61" spans="3:11" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
       <c r="E61" s="3"/>
@@ -2525,7 +4159,7 @@
       <c r="J61" s="3"/>
       <c r="K61" s="3"/>
     </row>
-    <row r="62" spans="3:11" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
       <c r="E62" s="3"/>
@@ -2536,7 +4170,7 @@
       <c r="J62" s="3"/>
       <c r="K62" s="3"/>
     </row>
-    <row r="63" spans="3:11" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
       <c r="E63" s="3"/>
@@ -2547,7 +4181,7 @@
       <c r="J63" s="3"/>
       <c r="K63" s="3"/>
     </row>
-    <row r="64" spans="3:11" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.2">
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>

</xml_diff>

<commit_message>
Added 5 new Entries
</commit_message>
<xml_diff>
--- a/assets/data/anime.xlsx
+++ b/assets/data/anime.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Anime Archive\assets\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68BDE85C-219D-49A6-B2E4-0A8239D1433D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{476ECD23-E9CE-4A80-87AD-7A4E6C4E7BCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-72" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Everything I Have Watched So Fa" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="364">
   <si>
     <t>Name</t>
   </si>
@@ -1037,6 +1037,81 @@
   </si>
   <si>
     <t>アーケイン (Ākein)</t>
+  </si>
+  <si>
+    <t>Love Unseen Beneath the Clear Night Sky</t>
+  </si>
+  <si>
+    <t>見えない恋は晴れた夜空のもとで (Mietenaishi Koi wa Hareta Yozora no Moto de)</t>
+  </si>
+  <si>
+    <t>Kei Oikawa</t>
+  </si>
+  <si>
+    <t>love-unseen-beneath-the-clear-night-sky</t>
+  </si>
+  <si>
+    <t>僕は彼女を勘違いしてる (Boku wa Kanojo wo Kanchigai Shiteru)</t>
+  </si>
+  <si>
+    <t>Pine Jam</t>
+  </si>
+  <si>
+    <t>Kazuhiro Yoneda</t>
+  </si>
+  <si>
+    <t>Comedy, Romance, Slice of Life</t>
+  </si>
+  <si>
+    <t>oh-boy-was-i-wrong-about-her</t>
+  </si>
+  <si>
+    <t>Oh Boy,  Was I Wrong About Her</t>
+  </si>
+  <si>
+    <t>I Want to Love You Till Your Dying Day</t>
+  </si>
+  <si>
+    <t>きみが死ぬまで恋をしたい (Kimi ga Shinu made Koi wo Shitai)</t>
+  </si>
+  <si>
+    <t>ROLL2</t>
+  </si>
+  <si>
+    <t>Yasushi Tomoda</t>
+  </si>
+  <si>
+    <t>Drama, Dark Fantasy, Yuri</t>
+  </si>
+  <si>
+    <t>i-want-to-love-you-till-your-dying-day</t>
+  </si>
+  <si>
+    <t>I Want to End This Love Game</t>
+  </si>
+  <si>
+    <t>愛してるゲームを終わらせたい (Aishiteiru Game wo Owarasetai)</t>
+  </si>
+  <si>
+    <t>Shota Umehara</t>
+  </si>
+  <si>
+    <t>i-want-to-end-this-love-game</t>
+  </si>
+  <si>
+    <t>Lycoris Recoil</t>
+  </si>
+  <si>
+    <t>リコリス・リコイル (Rikoris Rikoiru)</t>
+  </si>
+  <si>
+    <t>Shingo Adachi</t>
+  </si>
+  <si>
+    <t>Action, Sci-Fi</t>
+  </si>
+  <si>
+    <t>lycoris-recoil</t>
   </si>
 </sst>
 </file>
@@ -4136,59 +4211,245 @@
       </c>
     </row>
     <row r="58" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="C58" s="3"/>
-      <c r="D58" s="3"/>
-      <c r="E58" s="3"/>
+      <c r="A58" t="s">
+        <v>339</v>
+      </c>
+      <c r="B58" t="s">
+        <v>340</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D58" s="3">
+        <v>7.68</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>145</v>
+      </c>
       <c r="F58" s="3"/>
-      <c r="G58" s="3"/>
-      <c r="H58" s="3"/>
-      <c r="I58" s="3"/>
-      <c r="J58" s="3"/>
-      <c r="K58" s="3"/>
+      <c r="G58" s="3">
+        <v>1</v>
+      </c>
+      <c r="H58" s="3">
+        <v>12</v>
+      </c>
+      <c r="I58" s="3">
+        <v>2026</v>
+      </c>
+      <c r="J58" s="3">
+        <v>24</v>
+      </c>
+      <c r="K58" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="L58" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="M58" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="N58" s="4">
+        <v>57</v>
+      </c>
+      <c r="O58" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="Q58" s="4" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="59" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="C59" s="3"/>
-      <c r="D59" s="3"/>
-      <c r="E59" s="3"/>
+      <c r="A59" t="s">
+        <v>348</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D59" s="3">
+        <v>7.42</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>145</v>
+      </c>
       <c r="F59" s="3"/>
-      <c r="G59" s="3"/>
-      <c r="H59" s="3"/>
-      <c r="I59" s="3"/>
-      <c r="J59" s="3"/>
-      <c r="K59" s="3"/>
+      <c r="G59" s="3">
+        <v>1</v>
+      </c>
+      <c r="H59" s="3">
+        <v>12</v>
+      </c>
+      <c r="I59" s="3">
+        <v>2026</v>
+      </c>
+      <c r="J59" s="3">
+        <v>24</v>
+      </c>
+      <c r="K59" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="L59" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="M59" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="N59" s="4">
+        <v>58</v>
+      </c>
+      <c r="O59" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="P59" s="4"/>
+      <c r="Q59" s="4" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="60" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="C60" s="3"/>
-      <c r="D60" s="3"/>
-      <c r="E60" s="3"/>
+      <c r="A60" t="s">
+        <v>349</v>
+      </c>
+      <c r="B60" t="s">
+        <v>350</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D60" s="3">
+        <v>7.82</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>145</v>
+      </c>
       <c r="F60" s="3"/>
-      <c r="G60" s="3"/>
-      <c r="H60" s="3"/>
-      <c r="I60" s="3"/>
-      <c r="J60" s="3"/>
-      <c r="K60" s="3"/>
+      <c r="G60" s="3">
+        <v>1</v>
+      </c>
+      <c r="H60" s="3">
+        <v>12</v>
+      </c>
+      <c r="I60" s="3">
+        <v>2026</v>
+      </c>
+      <c r="J60" s="3">
+        <v>24</v>
+      </c>
+      <c r="K60" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="L60" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="M60" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="N60" s="4">
+        <v>59</v>
+      </c>
+      <c r="O60" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="Q60" s="4" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="61" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="C61" s="3"/>
-      <c r="D61" s="3"/>
-      <c r="E61" s="3"/>
+      <c r="A61" t="s">
+        <v>355</v>
+      </c>
+      <c r="B61" t="s">
+        <v>356</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D61" s="3">
+        <v>7.95</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>145</v>
+      </c>
       <c r="F61" s="3"/>
-      <c r="G61" s="3"/>
-      <c r="H61" s="3"/>
-      <c r="I61" s="3"/>
-      <c r="J61" s="3"/>
-      <c r="K61" s="3"/>
+      <c r="G61" s="3">
+        <v>1</v>
+      </c>
+      <c r="H61" s="3">
+        <v>12</v>
+      </c>
+      <c r="I61" s="3">
+        <v>2026</v>
+      </c>
+      <c r="J61" s="3">
+        <v>24</v>
+      </c>
+      <c r="K61" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="L61" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="M61" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="N61" s="4">
+        <v>60</v>
+      </c>
+      <c r="O61" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="Q61" s="4" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="62" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="C62" s="3"/>
-      <c r="D62" s="3"/>
-      <c r="E62" s="3"/>
+      <c r="A62" t="s">
+        <v>359</v>
+      </c>
+      <c r="B62" t="s">
+        <v>360</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D62" s="3">
+        <v>8.23</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>145</v>
+      </c>
       <c r="F62" s="3"/>
-      <c r="G62" s="3"/>
-      <c r="H62" s="3"/>
-      <c r="I62" s="3"/>
-      <c r="J62" s="3"/>
-      <c r="K62" s="3"/>
+      <c r="G62" s="3">
+        <v>1</v>
+      </c>
+      <c r="H62" s="3">
+        <v>13</v>
+      </c>
+      <c r="I62" s="3">
+        <v>2022</v>
+      </c>
+      <c r="J62" s="3">
+        <v>24</v>
+      </c>
+      <c r="K62" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="L62" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="M62" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="N62" s="4">
+        <v>61</v>
+      </c>
+      <c r="O62" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="Q62" s="4" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="63" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
       <c r="C63" s="3"/>

</xml_diff>

<commit_message>
Updated Silent Voice Data
</commit_message>
<xml_diff>
--- a/assets/data/anime.xlsx
+++ b/assets/data/anime.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Anime Archive\assets\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A41953-1B30-4BBD-9E9E-56E6F1E2DED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CF0E850-F746-4B18-A731-C30503F9DD04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2533,7 +2533,7 @@
         <v>151</v>
       </c>
       <c r="Q22" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="R22" s="4" t="s">
         <v>144</v>

</xml_diff>